<commit_message>
feat: agregar campo nee_comments en formulario y planilla de alumnos
- StudentProfileFormFields: nuevo campo "Comentarios NEE" (multiline)
  visible únicamente cuando NEE = Sí
- StudentProfileCreateForm y StudentProfileUpdateForm: nee_comments
  agregado a defaultValues (vacío al crear, precargado al editar)
- types.ts: nee_comments agregado como opcional a I_StudentProfileDetail
  e I_StudentProfileCreateRequestData
- Meta--PlanillaBaseAlumnos.xlsx: nueva columna "Comentarios NEE" con el
  mismo estilo de encabezado que las columnas existentes

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Meta--PlanillaBaseAlumnos.xlsx
+++ b/public/Meta--PlanillaBaseAlumnos.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -377,7 +377,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C501"/>
+  <dimension ref="A1:D501"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="20" customWidth="1" style="3" min="1" max="2"/>
@@ -401,11 +401,16 @@
           <t>NEE</t>
         </is>
       </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Comentarios NEE</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15.75" customHeight="1" s="3">
       <c r="A2" s="2" t="n"/>
       <c r="B2" s="2" t="n"/>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -414,7 +419,7 @@
     <row r="3" ht="15.75" customHeight="1" s="3">
       <c r="A3" s="2" t="n"/>
       <c r="B3" s="2" t="n"/>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -423,7 +428,7 @@
     <row r="4" ht="15.75" customHeight="1" s="3">
       <c r="A4" s="2" t="n"/>
       <c r="B4" s="2" t="n"/>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -431,7 +436,7 @@
     </row>
     <row r="5" ht="15.75" customHeight="1" s="3">
       <c r="B5" s="2" t="n"/>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -439,3472 +444,3472 @@
     </row>
     <row r="6" ht="15.75" customHeight="1" s="3">
       <c r="B6" s="2" t="n"/>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="3">
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="3">
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="3">
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="3">
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="3">
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="3">
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1" s="3">
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1" s="3">
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="3">
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1" s="3">
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1" s="3">
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1" s="3">
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1" s="3">
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="3">
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="3">
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="3">
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="3">
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="3">
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="3">
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="3">
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="3">
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="3">
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="3">
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="3">
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="3">
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="3">
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="3">
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="3">
-      <c r="C34" t="inlineStr">
+      <c r="C34" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="3">
-      <c r="C35" t="inlineStr">
+      <c r="C35" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="3">
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="3">
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="3">
-      <c r="C38" t="inlineStr">
+      <c r="C38" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="3">
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="3">
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="3">
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="3">
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="3">
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="3">
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="3">
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="3">
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="3">
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="3">
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="3">
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="3">
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="3">
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="3">
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="3">
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="3">
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="3">
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="3">
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="3">
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="3">
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="3">
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="3">
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="3">
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1" s="3">
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1" s="3">
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1" s="3">
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1" s="3">
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1" s="3">
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1" s="3">
-      <c r="C67" t="inlineStr">
+      <c r="C67" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1" s="3">
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1" s="3">
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1" s="3">
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1" s="3">
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15.75" customHeight="1" s="3">
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1" s="3">
-      <c r="C73" t="inlineStr">
+      <c r="C73" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1" s="3">
-      <c r="C74" t="inlineStr">
+      <c r="C74" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1" s="3">
-      <c r="C75" t="inlineStr">
+      <c r="C75" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15.75" customHeight="1" s="3">
-      <c r="C76" t="inlineStr">
+      <c r="C76" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15.75" customHeight="1" s="3">
-      <c r="C77" t="inlineStr">
+      <c r="C77" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1" s="3">
-      <c r="C78" t="inlineStr">
+      <c r="C78" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1" s="3">
-      <c r="C79" t="inlineStr">
+      <c r="C79" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1" s="3">
-      <c r="C80" t="inlineStr">
+      <c r="C80" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1" s="3">
-      <c r="C81" t="inlineStr">
+      <c r="C81" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15.75" customHeight="1" s="3">
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15.75" customHeight="1" s="3">
-      <c r="C83" t="inlineStr">
+      <c r="C83" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1" s="3">
-      <c r="C84" t="inlineStr">
+      <c r="C84" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15.75" customHeight="1" s="3">
-      <c r="C85" t="inlineStr">
+      <c r="C85" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15.75" customHeight="1" s="3">
-      <c r="C86" t="inlineStr">
+      <c r="C86" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15.75" customHeight="1" s="3">
-      <c r="C87" t="inlineStr">
+      <c r="C87" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15.75" customHeight="1" s="3">
-      <c r="C88" t="inlineStr">
+      <c r="C88" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15.75" customHeight="1" s="3">
-      <c r="C89" t="inlineStr">
+      <c r="C89" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15.75" customHeight="1" s="3">
-      <c r="C90" t="inlineStr">
+      <c r="C90" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15.75" customHeight="1" s="3">
-      <c r="C91" t="inlineStr">
+      <c r="C91" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1" s="3">
-      <c r="C92" t="inlineStr">
+      <c r="C92" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15.75" customHeight="1" s="3">
-      <c r="C93" t="inlineStr">
+      <c r="C93" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15.75" customHeight="1" s="3">
-      <c r="C94" t="inlineStr">
+      <c r="C94" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15.75" customHeight="1" s="3">
-      <c r="C95" t="inlineStr">
+      <c r="C95" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15.75" customHeight="1" s="3">
-      <c r="C96" t="inlineStr">
+      <c r="C96" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15.75" customHeight="1" s="3">
-      <c r="C97" t="inlineStr">
+      <c r="C97" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1" s="3">
-      <c r="C98" t="inlineStr">
+      <c r="C98" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15.75" customHeight="1" s="3">
-      <c r="C99" t="inlineStr">
+      <c r="C99" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15.75" customHeight="1" s="3">
-      <c r="C100" t="inlineStr">
+      <c r="C100" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15.75" customHeight="1" s="3">
-      <c r="C101" t="inlineStr">
+      <c r="C101" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15.75" customHeight="1" s="3">
-      <c r="C102" t="inlineStr">
+      <c r="C102" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15.75" customHeight="1" s="3">
-      <c r="C103" t="inlineStr">
+      <c r="C103" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="104" ht="15.75" customHeight="1" s="3">
-      <c r="C104" t="inlineStr">
+      <c r="C104" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="105" ht="15.75" customHeight="1" s="3">
-      <c r="C105" t="inlineStr">
+      <c r="C105" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="106" ht="15.75" customHeight="1" s="3">
-      <c r="C106" t="inlineStr">
+      <c r="C106" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15.75" customHeight="1" s="3">
-      <c r="C107" t="inlineStr">
+      <c r="C107" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="108" ht="15.75" customHeight="1" s="3">
-      <c r="C108" t="inlineStr">
+      <c r="C108" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15.75" customHeight="1" s="3">
-      <c r="C109" t="inlineStr">
+      <c r="C109" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15.75" customHeight="1" s="3">
-      <c r="C110" t="inlineStr">
+      <c r="C110" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="111" ht="15.75" customHeight="1" s="3">
-      <c r="C111" t="inlineStr">
+      <c r="C111" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="112" ht="15.75" customHeight="1" s="3">
-      <c r="C112" t="inlineStr">
+      <c r="C112" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="113" ht="15.75" customHeight="1" s="3">
-      <c r="C113" t="inlineStr">
+      <c r="C113" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="114" ht="15.75" customHeight="1" s="3">
-      <c r="C114" t="inlineStr">
+      <c r="C114" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="115" ht="15.75" customHeight="1" s="3">
-      <c r="C115" t="inlineStr">
+      <c r="C115" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="116" ht="15.75" customHeight="1" s="3">
-      <c r="C116" t="inlineStr">
+      <c r="C116" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="117" ht="15.75" customHeight="1" s="3">
-      <c r="C117" t="inlineStr">
+      <c r="C117" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="118" ht="15.75" customHeight="1" s="3">
-      <c r="C118" t="inlineStr">
+      <c r="C118" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="119" ht="15.75" customHeight="1" s="3">
-      <c r="C119" t="inlineStr">
+      <c r="C119" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="120" ht="15.75" customHeight="1" s="3">
-      <c r="C120" t="inlineStr">
+      <c r="C120" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="121" ht="15.75" customHeight="1" s="3">
-      <c r="C121" t="inlineStr">
+      <c r="C121" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="122" ht="15.75" customHeight="1" s="3">
-      <c r="C122" t="inlineStr">
+      <c r="C122" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="123" ht="15.75" customHeight="1" s="3">
-      <c r="C123" t="inlineStr">
+      <c r="C123" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="124" ht="15.75" customHeight="1" s="3">
-      <c r="C124" t="inlineStr">
+      <c r="C124" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="125" ht="15.75" customHeight="1" s="3">
-      <c r="C125" t="inlineStr">
+      <c r="C125" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="126" ht="15.75" customHeight="1" s="3">
-      <c r="C126" t="inlineStr">
+      <c r="C126" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="127" ht="15.75" customHeight="1" s="3">
-      <c r="C127" t="inlineStr">
+      <c r="C127" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="128" ht="15.75" customHeight="1" s="3">
-      <c r="C128" t="inlineStr">
+      <c r="C128" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="129" ht="15.75" customHeight="1" s="3">
-      <c r="C129" t="inlineStr">
+      <c r="C129" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="130" ht="15.75" customHeight="1" s="3">
-      <c r="C130" t="inlineStr">
+      <c r="C130" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="131" ht="15.75" customHeight="1" s="3">
-      <c r="C131" t="inlineStr">
+      <c r="C131" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="132" ht="15.75" customHeight="1" s="3">
-      <c r="C132" t="inlineStr">
+      <c r="C132" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="133" ht="15.75" customHeight="1" s="3">
-      <c r="C133" t="inlineStr">
+      <c r="C133" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="134" ht="15.75" customHeight="1" s="3">
-      <c r="C134" t="inlineStr">
+      <c r="C134" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="135" ht="15.75" customHeight="1" s="3">
-      <c r="C135" t="inlineStr">
+      <c r="C135" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="136" ht="15.75" customHeight="1" s="3">
-      <c r="C136" t="inlineStr">
+      <c r="C136" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="137" ht="15.75" customHeight="1" s="3">
-      <c r="C137" t="inlineStr">
+      <c r="C137" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="138" ht="15.75" customHeight="1" s="3">
-      <c r="C138" t="inlineStr">
+      <c r="C138" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="139" ht="15.75" customHeight="1" s="3">
-      <c r="C139" t="inlineStr">
+      <c r="C139" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="140" ht="15.75" customHeight="1" s="3">
-      <c r="C140" t="inlineStr">
+      <c r="C140" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="141" ht="15.75" customHeight="1" s="3">
-      <c r="C141" t="inlineStr">
+      <c r="C141" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="142" ht="15.75" customHeight="1" s="3">
-      <c r="C142" t="inlineStr">
+      <c r="C142" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="143" ht="15.75" customHeight="1" s="3">
-      <c r="C143" t="inlineStr">
+      <c r="C143" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="144" ht="15.75" customHeight="1" s="3">
-      <c r="C144" t="inlineStr">
+      <c r="C144" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="145" ht="15.75" customHeight="1" s="3">
-      <c r="C145" t="inlineStr">
+      <c r="C145" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="146" ht="15.75" customHeight="1" s="3">
-      <c r="C146" t="inlineStr">
+      <c r="C146" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="147" ht="15.75" customHeight="1" s="3">
-      <c r="C147" t="inlineStr">
+      <c r="C147" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="148" ht="15.75" customHeight="1" s="3">
-      <c r="C148" t="inlineStr">
+      <c r="C148" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="149" ht="15.75" customHeight="1" s="3">
-      <c r="C149" t="inlineStr">
+      <c r="C149" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="150" ht="15.75" customHeight="1" s="3">
-      <c r="C150" t="inlineStr">
+      <c r="C150" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="151" ht="15.75" customHeight="1" s="3">
-      <c r="C151" t="inlineStr">
+      <c r="C151" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="152" ht="15.75" customHeight="1" s="3">
-      <c r="C152" t="inlineStr">
+      <c r="C152" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="153" ht="15.75" customHeight="1" s="3">
-      <c r="C153" t="inlineStr">
+      <c r="C153" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="154" ht="15.75" customHeight="1" s="3">
-      <c r="C154" t="inlineStr">
+      <c r="C154" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="155" ht="15.75" customHeight="1" s="3">
-      <c r="C155" t="inlineStr">
+      <c r="C155" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="156" ht="15.75" customHeight="1" s="3">
-      <c r="C156" t="inlineStr">
+      <c r="C156" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="157" ht="15.75" customHeight="1" s="3">
-      <c r="C157" t="inlineStr">
+      <c r="C157" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="158" ht="15.75" customHeight="1" s="3">
-      <c r="C158" t="inlineStr">
+      <c r="C158" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="159" ht="15.75" customHeight="1" s="3">
-      <c r="C159" t="inlineStr">
+      <c r="C159" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="160" ht="15.75" customHeight="1" s="3">
-      <c r="C160" t="inlineStr">
+      <c r="C160" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="161" ht="15.75" customHeight="1" s="3">
-      <c r="C161" t="inlineStr">
+      <c r="C161" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="162" ht="15.75" customHeight="1" s="3">
-      <c r="C162" t="inlineStr">
+      <c r="C162" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="163" ht="15.75" customHeight="1" s="3">
-      <c r="C163" t="inlineStr">
+      <c r="C163" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="164" ht="15.75" customHeight="1" s="3">
-      <c r="C164" t="inlineStr">
+      <c r="C164" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="165" ht="15.75" customHeight="1" s="3">
-      <c r="C165" t="inlineStr">
+      <c r="C165" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="166" ht="15.75" customHeight="1" s="3">
-      <c r="C166" t="inlineStr">
+      <c r="C166" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="167" ht="15.75" customHeight="1" s="3">
-      <c r="C167" t="inlineStr">
+      <c r="C167" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="168" ht="15.75" customHeight="1" s="3">
-      <c r="C168" t="inlineStr">
+      <c r="C168" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="169" ht="15.75" customHeight="1" s="3">
-      <c r="C169" t="inlineStr">
+      <c r="C169" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="170" ht="15.75" customHeight="1" s="3">
-      <c r="C170" t="inlineStr">
+      <c r="C170" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="171" ht="15.75" customHeight="1" s="3">
-      <c r="C171" t="inlineStr">
+      <c r="C171" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="172" ht="15.75" customHeight="1" s="3">
-      <c r="C172" t="inlineStr">
+      <c r="C172" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="173" ht="15.75" customHeight="1" s="3">
-      <c r="C173" t="inlineStr">
+      <c r="C173" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="174" ht="15.75" customHeight="1" s="3">
-      <c r="C174" t="inlineStr">
+      <c r="C174" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="175" ht="15.75" customHeight="1" s="3">
-      <c r="C175" t="inlineStr">
+      <c r="C175" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="176" ht="15.75" customHeight="1" s="3">
-      <c r="C176" t="inlineStr">
+      <c r="C176" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="177" ht="15.75" customHeight="1" s="3">
-      <c r="C177" t="inlineStr">
+      <c r="C177" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="178" ht="15.75" customHeight="1" s="3">
-      <c r="C178" t="inlineStr">
+      <c r="C178" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="179" ht="15.75" customHeight="1" s="3">
-      <c r="C179" t="inlineStr">
+      <c r="C179" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="180" ht="15.75" customHeight="1" s="3">
-      <c r="C180" t="inlineStr">
+      <c r="C180" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="181" ht="15.75" customHeight="1" s="3">
-      <c r="C181" t="inlineStr">
+      <c r="C181" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="182" ht="15.75" customHeight="1" s="3">
-      <c r="C182" t="inlineStr">
+      <c r="C182" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="183" ht="15.75" customHeight="1" s="3">
-      <c r="C183" t="inlineStr">
+      <c r="C183" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="184" ht="15.75" customHeight="1" s="3">
-      <c r="C184" t="inlineStr">
+      <c r="C184" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="185" ht="15.75" customHeight="1" s="3">
-      <c r="C185" t="inlineStr">
+      <c r="C185" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="186" ht="15.75" customHeight="1" s="3">
-      <c r="C186" t="inlineStr">
+      <c r="C186" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="187" ht="15.75" customHeight="1" s="3">
-      <c r="C187" t="inlineStr">
+      <c r="C187" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="188" ht="15.75" customHeight="1" s="3">
-      <c r="C188" t="inlineStr">
+      <c r="C188" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="189" ht="15.75" customHeight="1" s="3">
-      <c r="C189" t="inlineStr">
+      <c r="C189" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="190" ht="15.75" customHeight="1" s="3">
-      <c r="C190" t="inlineStr">
+      <c r="C190" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="191" ht="15.75" customHeight="1" s="3">
-      <c r="C191" t="inlineStr">
+      <c r="C191" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="192" ht="15.75" customHeight="1" s="3">
-      <c r="C192" t="inlineStr">
+      <c r="C192" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="193" ht="15.75" customHeight="1" s="3">
-      <c r="C193" t="inlineStr">
+      <c r="C193" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="194" ht="15.75" customHeight="1" s="3">
-      <c r="C194" t="inlineStr">
+      <c r="C194" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="195" ht="15.75" customHeight="1" s="3">
-      <c r="C195" t="inlineStr">
+      <c r="C195" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="196" ht="15.75" customHeight="1" s="3">
-      <c r="C196" t="inlineStr">
+      <c r="C196" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="197" ht="15.75" customHeight="1" s="3">
-      <c r="C197" t="inlineStr">
+      <c r="C197" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="198" ht="15.75" customHeight="1" s="3">
-      <c r="C198" t="inlineStr">
+      <c r="C198" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="199" ht="15.75" customHeight="1" s="3">
-      <c r="C199" t="inlineStr">
+      <c r="C199" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="200" ht="15.75" customHeight="1" s="3">
-      <c r="C200" t="inlineStr">
+      <c r="C200" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="201" ht="15.75" customHeight="1" s="3">
-      <c r="C201" t="inlineStr">
+      <c r="C201" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="202" ht="15.75" customHeight="1" s="3">
-      <c r="C202" t="inlineStr">
+      <c r="C202" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="203" ht="15.75" customHeight="1" s="3">
-      <c r="C203" t="inlineStr">
+      <c r="C203" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="204" ht="15.75" customHeight="1" s="3">
-      <c r="C204" t="inlineStr">
+      <c r="C204" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="205" ht="15.75" customHeight="1" s="3">
-      <c r="C205" t="inlineStr">
+      <c r="C205" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="206" ht="15.75" customHeight="1" s="3">
-      <c r="C206" t="inlineStr">
+      <c r="C206" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="207" ht="15.75" customHeight="1" s="3">
-      <c r="C207" t="inlineStr">
+      <c r="C207" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="208" ht="15.75" customHeight="1" s="3">
-      <c r="C208" t="inlineStr">
+      <c r="C208" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="209" ht="15.75" customHeight="1" s="3">
-      <c r="C209" t="inlineStr">
+      <c r="C209" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="210" ht="15.75" customHeight="1" s="3">
-      <c r="C210" t="inlineStr">
+      <c r="C210" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="211" ht="15.75" customHeight="1" s="3">
-      <c r="C211" t="inlineStr">
+      <c r="C211" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="212" ht="15.75" customHeight="1" s="3">
-      <c r="C212" t="inlineStr">
+      <c r="C212" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="213" ht="15.75" customHeight="1" s="3">
-      <c r="C213" t="inlineStr">
+      <c r="C213" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="214" ht="15.75" customHeight="1" s="3">
-      <c r="C214" t="inlineStr">
+      <c r="C214" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="215" ht="15.75" customHeight="1" s="3">
-      <c r="C215" t="inlineStr">
+      <c r="C215" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="216" ht="15.75" customHeight="1" s="3">
-      <c r="C216" t="inlineStr">
+      <c r="C216" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="217" ht="15.75" customHeight="1" s="3">
-      <c r="C217" t="inlineStr">
+      <c r="C217" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="218" ht="15.75" customHeight="1" s="3">
-      <c r="C218" t="inlineStr">
+      <c r="C218" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="219" ht="15.75" customHeight="1" s="3">
-      <c r="C219" t="inlineStr">
+      <c r="C219" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="220" ht="15.75" customHeight="1" s="3">
-      <c r="C220" t="inlineStr">
+      <c r="C220" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="221" ht="15.75" customHeight="1" s="3">
-      <c r="C221" t="inlineStr">
+      <c r="C221" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="222" ht="15.75" customHeight="1" s="3">
-      <c r="C222" t="inlineStr">
+      <c r="C222" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="223" ht="15.75" customHeight="1" s="3">
-      <c r="C223" t="inlineStr">
+      <c r="C223" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="224" ht="15.75" customHeight="1" s="3">
-      <c r="C224" t="inlineStr">
+      <c r="C224" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="225" ht="15.75" customHeight="1" s="3">
-      <c r="C225" t="inlineStr">
+      <c r="C225" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="226" ht="15.75" customHeight="1" s="3">
-      <c r="C226" t="inlineStr">
+      <c r="C226" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="227" ht="15.75" customHeight="1" s="3">
-      <c r="C227" t="inlineStr">
+      <c r="C227" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="228" ht="15.75" customHeight="1" s="3">
-      <c r="C228" t="inlineStr">
+      <c r="C228" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="229" ht="15.75" customHeight="1" s="3">
-      <c r="C229" t="inlineStr">
+      <c r="C229" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="230" ht="15.75" customHeight="1" s="3">
-      <c r="C230" t="inlineStr">
+      <c r="C230" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="231" ht="15.75" customHeight="1" s="3">
-      <c r="C231" t="inlineStr">
+      <c r="C231" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="232" ht="15.75" customHeight="1" s="3">
-      <c r="C232" t="inlineStr">
+      <c r="C232" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="233" ht="15.75" customHeight="1" s="3">
-      <c r="C233" t="inlineStr">
+      <c r="C233" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="234" ht="15.75" customHeight="1" s="3">
-      <c r="C234" t="inlineStr">
+      <c r="C234" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="235" ht="15.75" customHeight="1" s="3">
-      <c r="C235" t="inlineStr">
+      <c r="C235" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="236" ht="15.75" customHeight="1" s="3">
-      <c r="C236" t="inlineStr">
+      <c r="C236" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="237" ht="15.75" customHeight="1" s="3">
-      <c r="C237" t="inlineStr">
+      <c r="C237" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="238" ht="15.75" customHeight="1" s="3">
-      <c r="C238" t="inlineStr">
+      <c r="C238" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="239" ht="15.75" customHeight="1" s="3">
-      <c r="C239" t="inlineStr">
+      <c r="C239" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="240" ht="15.75" customHeight="1" s="3">
-      <c r="C240" t="inlineStr">
+      <c r="C240" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="241" ht="15.75" customHeight="1" s="3">
-      <c r="C241" t="inlineStr">
+      <c r="C241" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="242" ht="15.75" customHeight="1" s="3">
-      <c r="C242" t="inlineStr">
+      <c r="C242" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="243" ht="15.75" customHeight="1" s="3">
-      <c r="C243" t="inlineStr">
+      <c r="C243" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="244" ht="15.75" customHeight="1" s="3">
-      <c r="C244" t="inlineStr">
+      <c r="C244" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="245" ht="15.75" customHeight="1" s="3">
-      <c r="C245" t="inlineStr">
+      <c r="C245" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="246" ht="15.75" customHeight="1" s="3">
-      <c r="C246" t="inlineStr">
+      <c r="C246" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="247" ht="15.75" customHeight="1" s="3">
-      <c r="C247" t="inlineStr">
+      <c r="C247" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="248" ht="15.75" customHeight="1" s="3">
-      <c r="C248" t="inlineStr">
+      <c r="C248" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="249" ht="15.75" customHeight="1" s="3">
-      <c r="C249" t="inlineStr">
+      <c r="C249" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="250" ht="15.75" customHeight="1" s="3">
-      <c r="C250" t="inlineStr">
+      <c r="C250" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="251" ht="15.75" customHeight="1" s="3">
-      <c r="C251" t="inlineStr">
+      <c r="C251" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="252" ht="15.75" customHeight="1" s="3">
-      <c r="C252" t="inlineStr">
+      <c r="C252" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="253" ht="15.75" customHeight="1" s="3">
-      <c r="C253" t="inlineStr">
+      <c r="C253" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="254" ht="15.75" customHeight="1" s="3">
-      <c r="C254" t="inlineStr">
+      <c r="C254" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="255" ht="15.75" customHeight="1" s="3">
-      <c r="C255" t="inlineStr">
+      <c r="C255" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="256" ht="15.75" customHeight="1" s="3">
-      <c r="C256" t="inlineStr">
+      <c r="C256" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="257" ht="15.75" customHeight="1" s="3">
-      <c r="C257" t="inlineStr">
+      <c r="C257" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="258" ht="15.75" customHeight="1" s="3">
-      <c r="C258" t="inlineStr">
+      <c r="C258" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="259" ht="15.75" customHeight="1" s="3">
-      <c r="C259" t="inlineStr">
+      <c r="C259" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="260" ht="15.75" customHeight="1" s="3">
-      <c r="C260" t="inlineStr">
+      <c r="C260" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="261" ht="15.75" customHeight="1" s="3">
-      <c r="C261" t="inlineStr">
+      <c r="C261" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="262" ht="15.75" customHeight="1" s="3">
-      <c r="C262" t="inlineStr">
+      <c r="C262" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="263" ht="15.75" customHeight="1" s="3">
-      <c r="C263" t="inlineStr">
+      <c r="C263" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="264" ht="15.75" customHeight="1" s="3">
-      <c r="C264" t="inlineStr">
+      <c r="C264" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="265" ht="15.75" customHeight="1" s="3">
-      <c r="C265" t="inlineStr">
+      <c r="C265" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="266" ht="15.75" customHeight="1" s="3">
-      <c r="C266" t="inlineStr">
+      <c r="C266" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="267" ht="15.75" customHeight="1" s="3">
-      <c r="C267" t="inlineStr">
+      <c r="C267" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="268" ht="15.75" customHeight="1" s="3">
-      <c r="C268" t="inlineStr">
+      <c r="C268" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="269" ht="15.75" customHeight="1" s="3">
-      <c r="C269" t="inlineStr">
+      <c r="C269" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="270" ht="15.75" customHeight="1" s="3">
-      <c r="C270" t="inlineStr">
+      <c r="C270" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="271" ht="15.75" customHeight="1" s="3">
-      <c r="C271" t="inlineStr">
+      <c r="C271" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="272" ht="15.75" customHeight="1" s="3">
-      <c r="C272" t="inlineStr">
+      <c r="C272" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="273" ht="15.75" customHeight="1" s="3">
-      <c r="C273" t="inlineStr">
+      <c r="C273" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="274" ht="15.75" customHeight="1" s="3">
-      <c r="C274" t="inlineStr">
+      <c r="C274" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="275" ht="15.75" customHeight="1" s="3">
-      <c r="C275" t="inlineStr">
+      <c r="C275" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="276" ht="15.75" customHeight="1" s="3">
-      <c r="C276" t="inlineStr">
+      <c r="C276" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="277" ht="15.75" customHeight="1" s="3">
-      <c r="C277" t="inlineStr">
+      <c r="C277" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="278" ht="15.75" customHeight="1" s="3">
-      <c r="C278" t="inlineStr">
+      <c r="C278" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="279" ht="15.75" customHeight="1" s="3">
-      <c r="C279" t="inlineStr">
+      <c r="C279" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="280" ht="15.75" customHeight="1" s="3">
-      <c r="C280" t="inlineStr">
+      <c r="C280" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="281" ht="15.75" customHeight="1" s="3">
-      <c r="C281" t="inlineStr">
+      <c r="C281" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="282" ht="15.75" customHeight="1" s="3">
-      <c r="C282" t="inlineStr">
+      <c r="C282" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="283" ht="15.75" customHeight="1" s="3">
-      <c r="C283" t="inlineStr">
+      <c r="C283" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="284" ht="15.75" customHeight="1" s="3">
-      <c r="C284" t="inlineStr">
+      <c r="C284" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="285" ht="15.75" customHeight="1" s="3">
-      <c r="C285" t="inlineStr">
+      <c r="C285" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="286" ht="15.75" customHeight="1" s="3">
-      <c r="C286" t="inlineStr">
+      <c r="C286" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="287" ht="15.75" customHeight="1" s="3">
-      <c r="C287" t="inlineStr">
+      <c r="C287" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="288" ht="15.75" customHeight="1" s="3">
-      <c r="C288" t="inlineStr">
+      <c r="C288" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="289" ht="15.75" customHeight="1" s="3">
-      <c r="C289" t="inlineStr">
+      <c r="C289" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="290" ht="15.75" customHeight="1" s="3">
-      <c r="C290" t="inlineStr">
+      <c r="C290" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="291" ht="15.75" customHeight="1" s="3">
-      <c r="C291" t="inlineStr">
+      <c r="C291" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="292" ht="15.75" customHeight="1" s="3">
-      <c r="C292" t="inlineStr">
+      <c r="C292" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="293" ht="15.75" customHeight="1" s="3">
-      <c r="C293" t="inlineStr">
+      <c r="C293" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="294" ht="15.75" customHeight="1" s="3">
-      <c r="C294" t="inlineStr">
+      <c r="C294" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="295" ht="15.75" customHeight="1" s="3">
-      <c r="C295" t="inlineStr">
+      <c r="C295" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="296" ht="15.75" customHeight="1" s="3">
-      <c r="C296" t="inlineStr">
+      <c r="C296" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="297" ht="15.75" customHeight="1" s="3">
-      <c r="C297" t="inlineStr">
+      <c r="C297" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="298" ht="15.75" customHeight="1" s="3">
-      <c r="C298" t="inlineStr">
+      <c r="C298" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="299" ht="15.75" customHeight="1" s="3">
-      <c r="C299" t="inlineStr">
+      <c r="C299" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="300" ht="15.75" customHeight="1" s="3">
-      <c r="C300" t="inlineStr">
+      <c r="C300" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="301" ht="15.75" customHeight="1" s="3">
-      <c r="C301" t="inlineStr">
+      <c r="C301" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="302" ht="15.75" customHeight="1" s="3">
-      <c r="C302" t="inlineStr">
+      <c r="C302" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="303" ht="15.75" customHeight="1" s="3">
-      <c r="C303" t="inlineStr">
+      <c r="C303" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="304" ht="15.75" customHeight="1" s="3">
-      <c r="C304" t="inlineStr">
+      <c r="C304" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="305" ht="15.75" customHeight="1" s="3">
-      <c r="C305" t="inlineStr">
+      <c r="C305" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="306" ht="15.75" customHeight="1" s="3">
-      <c r="C306" t="inlineStr">
+      <c r="C306" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="307" ht="15.75" customHeight="1" s="3">
-      <c r="C307" t="inlineStr">
+      <c r="C307" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="308" ht="15.75" customHeight="1" s="3">
-      <c r="C308" t="inlineStr">
+      <c r="C308" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="309" ht="15.75" customHeight="1" s="3">
-      <c r="C309" t="inlineStr">
+      <c r="C309" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="310" ht="15.75" customHeight="1" s="3">
-      <c r="C310" t="inlineStr">
+      <c r="C310" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="311" ht="15.75" customHeight="1" s="3">
-      <c r="C311" t="inlineStr">
+      <c r="C311" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="312" ht="15.75" customHeight="1" s="3">
-      <c r="C312" t="inlineStr">
+      <c r="C312" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="313" ht="15.75" customHeight="1" s="3">
-      <c r="C313" t="inlineStr">
+      <c r="C313" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="314" ht="15.75" customHeight="1" s="3">
-      <c r="C314" t="inlineStr">
+      <c r="C314" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="315" ht="15.75" customHeight="1" s="3">
-      <c r="C315" t="inlineStr">
+      <c r="C315" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="316" ht="15.75" customHeight="1" s="3">
-      <c r="C316" t="inlineStr">
+      <c r="C316" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="317" ht="15.75" customHeight="1" s="3">
-      <c r="C317" t="inlineStr">
+      <c r="C317" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="318" ht="15.75" customHeight="1" s="3">
-      <c r="C318" t="inlineStr">
+      <c r="C318" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="319" ht="15.75" customHeight="1" s="3">
-      <c r="C319" t="inlineStr">
+      <c r="C319" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="320" ht="15.75" customHeight="1" s="3">
-      <c r="C320" t="inlineStr">
+      <c r="C320" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="321" ht="15.75" customHeight="1" s="3">
-      <c r="C321" t="inlineStr">
+      <c r="C321" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="322" ht="15.75" customHeight="1" s="3">
-      <c r="C322" t="inlineStr">
+      <c r="C322" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="323" ht="15.75" customHeight="1" s="3">
-      <c r="C323" t="inlineStr">
+      <c r="C323" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="324" ht="15.75" customHeight="1" s="3">
-      <c r="C324" t="inlineStr">
+      <c r="C324" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="325" ht="15.75" customHeight="1" s="3">
-      <c r="C325" t="inlineStr">
+      <c r="C325" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="326" ht="15.75" customHeight="1" s="3">
-      <c r="C326" t="inlineStr">
+      <c r="C326" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="327" ht="15.75" customHeight="1" s="3">
-      <c r="C327" t="inlineStr">
+      <c r="C327" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="328" ht="15.75" customHeight="1" s="3">
-      <c r="C328" t="inlineStr">
+      <c r="C328" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="329" ht="15.75" customHeight="1" s="3">
-      <c r="C329" t="inlineStr">
+      <c r="C329" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="330" ht="15.75" customHeight="1" s="3">
-      <c r="C330" t="inlineStr">
+      <c r="C330" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="331" ht="15.75" customHeight="1" s="3">
-      <c r="C331" t="inlineStr">
+      <c r="C331" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="332" ht="15.75" customHeight="1" s="3">
-      <c r="C332" t="inlineStr">
+      <c r="C332" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="333" ht="15.75" customHeight="1" s="3">
-      <c r="C333" t="inlineStr">
+      <c r="C333" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="334" ht="15.75" customHeight="1" s="3">
-      <c r="C334" t="inlineStr">
+      <c r="C334" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="335" ht="15.75" customHeight="1" s="3">
-      <c r="C335" t="inlineStr">
+      <c r="C335" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="336" ht="15.75" customHeight="1" s="3">
-      <c r="C336" t="inlineStr">
+      <c r="C336" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="337" ht="15.75" customHeight="1" s="3">
-      <c r="C337" t="inlineStr">
+      <c r="C337" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="338" ht="15.75" customHeight="1" s="3">
-      <c r="C338" t="inlineStr">
+      <c r="C338" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="339" ht="15.75" customHeight="1" s="3">
-      <c r="C339" t="inlineStr">
+      <c r="C339" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="340" ht="15.75" customHeight="1" s="3">
-      <c r="C340" t="inlineStr">
+      <c r="C340" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="341" ht="15.75" customHeight="1" s="3">
-      <c r="C341" t="inlineStr">
+      <c r="C341" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="342" ht="15.75" customHeight="1" s="3">
-      <c r="C342" t="inlineStr">
+      <c r="C342" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="343" ht="15.75" customHeight="1" s="3">
-      <c r="C343" t="inlineStr">
+      <c r="C343" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="344" ht="15.75" customHeight="1" s="3">
-      <c r="C344" t="inlineStr">
+      <c r="C344" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="345" ht="15.75" customHeight="1" s="3">
-      <c r="C345" t="inlineStr">
+      <c r="C345" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="346" ht="15.75" customHeight="1" s="3">
-      <c r="C346" t="inlineStr">
+      <c r="C346" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="347" ht="15.75" customHeight="1" s="3">
-      <c r="C347" t="inlineStr">
+      <c r="C347" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="348" ht="15.75" customHeight="1" s="3">
-      <c r="C348" t="inlineStr">
+      <c r="C348" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="349" ht="15.75" customHeight="1" s="3">
-      <c r="C349" t="inlineStr">
+      <c r="C349" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="350" ht="15.75" customHeight="1" s="3">
-      <c r="C350" t="inlineStr">
+      <c r="C350" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="351" ht="15.75" customHeight="1" s="3">
-      <c r="C351" t="inlineStr">
+      <c r="C351" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="352" ht="15.75" customHeight="1" s="3">
-      <c r="C352" t="inlineStr">
+      <c r="C352" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="353" ht="15.75" customHeight="1" s="3">
-      <c r="C353" t="inlineStr">
+      <c r="C353" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="354" ht="15.75" customHeight="1" s="3">
-      <c r="C354" t="inlineStr">
+      <c r="C354" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="355" ht="15.75" customHeight="1" s="3">
-      <c r="C355" t="inlineStr">
+      <c r="C355" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="356" ht="15.75" customHeight="1" s="3">
-      <c r="C356" t="inlineStr">
+      <c r="C356" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="357" ht="15.75" customHeight="1" s="3">
-      <c r="C357" t="inlineStr">
+      <c r="C357" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="358" ht="15.75" customHeight="1" s="3">
-      <c r="C358" t="inlineStr">
+      <c r="C358" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="359" ht="15.75" customHeight="1" s="3">
-      <c r="C359" t="inlineStr">
+      <c r="C359" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="360" ht="15.75" customHeight="1" s="3">
-      <c r="C360" t="inlineStr">
+      <c r="C360" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="361" ht="15.75" customHeight="1" s="3">
-      <c r="C361" t="inlineStr">
+      <c r="C361" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="362" ht="15.75" customHeight="1" s="3">
-      <c r="C362" t="inlineStr">
+      <c r="C362" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="363" ht="15.75" customHeight="1" s="3">
-      <c r="C363" t="inlineStr">
+      <c r="C363" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="364" ht="15.75" customHeight="1" s="3">
-      <c r="C364" t="inlineStr">
+      <c r="C364" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="365" ht="15.75" customHeight="1" s="3">
-      <c r="C365" t="inlineStr">
+      <c r="C365" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="366" ht="15.75" customHeight="1" s="3">
-      <c r="C366" t="inlineStr">
+      <c r="C366" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="367" ht="15.75" customHeight="1" s="3">
-      <c r="C367" t="inlineStr">
+      <c r="C367" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="368" ht="15.75" customHeight="1" s="3">
-      <c r="C368" t="inlineStr">
+      <c r="C368" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="369" ht="15.75" customHeight="1" s="3">
-      <c r="C369" t="inlineStr">
+      <c r="C369" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="370" ht="15.75" customHeight="1" s="3">
-      <c r="C370" t="inlineStr">
+      <c r="C370" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="371" ht="15.75" customHeight="1" s="3">
-      <c r="C371" t="inlineStr">
+      <c r="C371" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="372" ht="15.75" customHeight="1" s="3">
-      <c r="C372" t="inlineStr">
+      <c r="C372" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="373" ht="15.75" customHeight="1" s="3">
-      <c r="C373" t="inlineStr">
+      <c r="C373" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="374" ht="15.75" customHeight="1" s="3">
-      <c r="C374" t="inlineStr">
+      <c r="C374" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="375" ht="15.75" customHeight="1" s="3">
-      <c r="C375" t="inlineStr">
+      <c r="C375" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="376" ht="15.75" customHeight="1" s="3">
-      <c r="C376" t="inlineStr">
+      <c r="C376" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="377" ht="15.75" customHeight="1" s="3">
-      <c r="C377" t="inlineStr">
+      <c r="C377" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="378" ht="15.75" customHeight="1" s="3">
-      <c r="C378" t="inlineStr">
+      <c r="C378" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="379" ht="15.75" customHeight="1" s="3">
-      <c r="C379" t="inlineStr">
+      <c r="C379" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="380" ht="15.75" customHeight="1" s="3">
-      <c r="C380" t="inlineStr">
+      <c r="C380" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="381" ht="15.75" customHeight="1" s="3">
-      <c r="C381" t="inlineStr">
+      <c r="C381" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="382" ht="15.75" customHeight="1" s="3">
-      <c r="C382" t="inlineStr">
+      <c r="C382" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="383" ht="15.75" customHeight="1" s="3">
-      <c r="C383" t="inlineStr">
+      <c r="C383" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="384" ht="15.75" customHeight="1" s="3">
-      <c r="C384" t="inlineStr">
+      <c r="C384" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="385" ht="15.75" customHeight="1" s="3">
-      <c r="C385" t="inlineStr">
+      <c r="C385" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="386" ht="15.75" customHeight="1" s="3">
-      <c r="C386" t="inlineStr">
+      <c r="C386" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="387" ht="15.75" customHeight="1" s="3">
-      <c r="C387" t="inlineStr">
+      <c r="C387" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="388" ht="15.75" customHeight="1" s="3">
-      <c r="C388" t="inlineStr">
+      <c r="C388" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="389" ht="15.75" customHeight="1" s="3">
-      <c r="C389" t="inlineStr">
+      <c r="C389" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="390" ht="15.75" customHeight="1" s="3">
-      <c r="C390" t="inlineStr">
+      <c r="C390" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="391" ht="15.75" customHeight="1" s="3">
-      <c r="C391" t="inlineStr">
+      <c r="C391" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="392" ht="15.75" customHeight="1" s="3">
-      <c r="C392" t="inlineStr">
+      <c r="C392" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="393" ht="15.75" customHeight="1" s="3">
-      <c r="C393" t="inlineStr">
+      <c r="C393" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="394" ht="15.75" customHeight="1" s="3">
-      <c r="C394" t="inlineStr">
+      <c r="C394" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="395" ht="15.75" customHeight="1" s="3">
-      <c r="C395" t="inlineStr">
+      <c r="C395" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="396" ht="15.75" customHeight="1" s="3">
-      <c r="C396" t="inlineStr">
+      <c r="C396" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="397" ht="15.75" customHeight="1" s="3">
-      <c r="C397" t="inlineStr">
+      <c r="C397" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="398" ht="15.75" customHeight="1" s="3">
-      <c r="C398" t="inlineStr">
+      <c r="C398" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="399" ht="15.75" customHeight="1" s="3">
-      <c r="C399" t="inlineStr">
+      <c r="C399" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="400" ht="15.75" customHeight="1" s="3">
-      <c r="C400" t="inlineStr">
+      <c r="C400" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="401" ht="15.75" customHeight="1" s="3">
-      <c r="C401" t="inlineStr">
+      <c r="C401" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="402" ht="15.75" customHeight="1" s="3">
-      <c r="C402" t="inlineStr">
+      <c r="C402" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="403" ht="15.75" customHeight="1" s="3">
-      <c r="C403" t="inlineStr">
+      <c r="C403" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="404" ht="15.75" customHeight="1" s="3">
-      <c r="C404" t="inlineStr">
+      <c r="C404" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="405" ht="15.75" customHeight="1" s="3">
-      <c r="C405" t="inlineStr">
+      <c r="C405" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="406" ht="15.75" customHeight="1" s="3">
-      <c r="C406" t="inlineStr">
+      <c r="C406" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="407" ht="15.75" customHeight="1" s="3">
-      <c r="C407" t="inlineStr">
+      <c r="C407" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="408" ht="15.75" customHeight="1" s="3">
-      <c r="C408" t="inlineStr">
+      <c r="C408" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="409" ht="15.75" customHeight="1" s="3">
-      <c r="C409" t="inlineStr">
+      <c r="C409" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="410" ht="15.75" customHeight="1" s="3">
-      <c r="C410" t="inlineStr">
+      <c r="C410" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="411" ht="15.75" customHeight="1" s="3">
-      <c r="C411" t="inlineStr">
+      <c r="C411" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="412" ht="15.75" customHeight="1" s="3">
-      <c r="C412" t="inlineStr">
+      <c r="C412" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="413" ht="15.75" customHeight="1" s="3">
-      <c r="C413" t="inlineStr">
+      <c r="C413" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="414" ht="15.75" customHeight="1" s="3">
-      <c r="C414" t="inlineStr">
+      <c r="C414" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="415" ht="15.75" customHeight="1" s="3">
-      <c r="C415" t="inlineStr">
+      <c r="C415" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="416" ht="15.75" customHeight="1" s="3">
-      <c r="C416" t="inlineStr">
+      <c r="C416" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="417" ht="15.75" customHeight="1" s="3">
-      <c r="C417" t="inlineStr">
+      <c r="C417" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="418" ht="15.75" customHeight="1" s="3">
-      <c r="C418" t="inlineStr">
+      <c r="C418" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="419" ht="15.75" customHeight="1" s="3">
-      <c r="C419" t="inlineStr">
+      <c r="C419" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="420" ht="15.75" customHeight="1" s="3">
-      <c r="C420" t="inlineStr">
+      <c r="C420" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="421" ht="15.75" customHeight="1" s="3">
-      <c r="C421" t="inlineStr">
+      <c r="C421" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="422" ht="15.75" customHeight="1" s="3">
-      <c r="C422" t="inlineStr">
+      <c r="C422" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="423" ht="15.75" customHeight="1" s="3">
-      <c r="C423" t="inlineStr">
+      <c r="C423" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="424" ht="15.75" customHeight="1" s="3">
-      <c r="C424" t="inlineStr">
+      <c r="C424" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="425" ht="15.75" customHeight="1" s="3">
-      <c r="C425" t="inlineStr">
+      <c r="C425" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="426" ht="15.75" customHeight="1" s="3">
-      <c r="C426" t="inlineStr">
+      <c r="C426" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="427" ht="15.75" customHeight="1" s="3">
-      <c r="C427" t="inlineStr">
+      <c r="C427" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="428" ht="15.75" customHeight="1" s="3">
-      <c r="C428" t="inlineStr">
+      <c r="C428" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="429" ht="15.75" customHeight="1" s="3">
-      <c r="C429" t="inlineStr">
+      <c r="C429" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="430" ht="15.75" customHeight="1" s="3">
-      <c r="C430" t="inlineStr">
+      <c r="C430" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="431" ht="15.75" customHeight="1" s="3">
-      <c r="C431" t="inlineStr">
+      <c r="C431" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="432" ht="15.75" customHeight="1" s="3">
-      <c r="C432" t="inlineStr">
+      <c r="C432" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="433" ht="15.75" customHeight="1" s="3">
-      <c r="C433" t="inlineStr">
+      <c r="C433" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="434" ht="15.75" customHeight="1" s="3">
-      <c r="C434" t="inlineStr">
+      <c r="C434" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="435" ht="15.75" customHeight="1" s="3">
-      <c r="C435" t="inlineStr">
+      <c r="C435" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="436" ht="15.75" customHeight="1" s="3">
-      <c r="C436" t="inlineStr">
+      <c r="C436" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="437" ht="15.75" customHeight="1" s="3">
-      <c r="C437" t="inlineStr">
+      <c r="C437" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="438" ht="15.75" customHeight="1" s="3">
-      <c r="C438" t="inlineStr">
+      <c r="C438" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="439" ht="15.75" customHeight="1" s="3">
-      <c r="C439" t="inlineStr">
+      <c r="C439" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="440" ht="15.75" customHeight="1" s="3">
-      <c r="C440" t="inlineStr">
+      <c r="C440" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="441" ht="15.75" customHeight="1" s="3">
-      <c r="C441" t="inlineStr">
+      <c r="C441" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="442" ht="15.75" customHeight="1" s="3">
-      <c r="C442" t="inlineStr">
+      <c r="C442" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="443" ht="15.75" customHeight="1" s="3">
-      <c r="C443" t="inlineStr">
+      <c r="C443" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="444" ht="15.75" customHeight="1" s="3">
-      <c r="C444" t="inlineStr">
+      <c r="C444" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="445" ht="15.75" customHeight="1" s="3">
-      <c r="C445" t="inlineStr">
+      <c r="C445" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="446" ht="15.75" customHeight="1" s="3">
-      <c r="C446" t="inlineStr">
+      <c r="C446" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="447" ht="15.75" customHeight="1" s="3">
-      <c r="C447" t="inlineStr">
+      <c r="C447" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="448" ht="15.75" customHeight="1" s="3">
-      <c r="C448" t="inlineStr">
+      <c r="C448" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="449" ht="15.75" customHeight="1" s="3">
-      <c r="C449" t="inlineStr">
+      <c r="C449" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="450" ht="15.75" customHeight="1" s="3">
-      <c r="C450" t="inlineStr">
+      <c r="C450" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="451" ht="15.75" customHeight="1" s="3">
-      <c r="C451" t="inlineStr">
+      <c r="C451" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="452" ht="15.75" customHeight="1" s="3">
-      <c r="C452" t="inlineStr">
+      <c r="C452" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="453" ht="15.75" customHeight="1" s="3">
-      <c r="C453" t="inlineStr">
+      <c r="C453" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="454" ht="15.75" customHeight="1" s="3">
-      <c r="C454" t="inlineStr">
+      <c r="C454" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="455" ht="15.75" customHeight="1" s="3">
-      <c r="C455" t="inlineStr">
+      <c r="C455" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="456" ht="15.75" customHeight="1" s="3">
-      <c r="C456" t="inlineStr">
+      <c r="C456" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="457" ht="15.75" customHeight="1" s="3">
-      <c r="C457" t="inlineStr">
+      <c r="C457" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="458" ht="15.75" customHeight="1" s="3">
-      <c r="C458" t="inlineStr">
+      <c r="C458" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="459" ht="15.75" customHeight="1" s="3">
-      <c r="C459" t="inlineStr">
+      <c r="C459" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="460" ht="15.75" customHeight="1" s="3">
-      <c r="C460" t="inlineStr">
+      <c r="C460" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="461" ht="15.75" customHeight="1" s="3">
-      <c r="C461" t="inlineStr">
+      <c r="C461" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="462" ht="15.75" customHeight="1" s="3">
-      <c r="C462" t="inlineStr">
+      <c r="C462" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="463" ht="15.75" customHeight="1" s="3">
-      <c r="C463" t="inlineStr">
+      <c r="C463" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="464" ht="15.75" customHeight="1" s="3">
-      <c r="C464" t="inlineStr">
+      <c r="C464" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="465" ht="15.75" customHeight="1" s="3">
-      <c r="C465" t="inlineStr">
+      <c r="C465" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="466" ht="15.75" customHeight="1" s="3">
-      <c r="C466" t="inlineStr">
+      <c r="C466" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="467" ht="15.75" customHeight="1" s="3">
-      <c r="C467" t="inlineStr">
+      <c r="C467" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="468" ht="15.75" customHeight="1" s="3">
-      <c r="C468" t="inlineStr">
+      <c r="C468" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="469" ht="15.75" customHeight="1" s="3">
-      <c r="C469" t="inlineStr">
+      <c r="C469" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="470" ht="15.75" customHeight="1" s="3">
-      <c r="C470" t="inlineStr">
+      <c r="C470" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="471" ht="15.75" customHeight="1" s="3">
-      <c r="C471" t="inlineStr">
+      <c r="C471" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="472" ht="15.75" customHeight="1" s="3">
-      <c r="C472" t="inlineStr">
+      <c r="C472" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="473" ht="15.75" customHeight="1" s="3">
-      <c r="C473" t="inlineStr">
+      <c r="C473" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="474" ht="15.75" customHeight="1" s="3">
-      <c r="C474" t="inlineStr">
+      <c r="C474" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="475" ht="15.75" customHeight="1" s="3">
-      <c r="C475" t="inlineStr">
+      <c r="C475" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="476" ht="15.75" customHeight="1" s="3">
-      <c r="C476" t="inlineStr">
+      <c r="C476" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="477" ht="15.75" customHeight="1" s="3">
-      <c r="C477" t="inlineStr">
+      <c r="C477" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="478" ht="15.75" customHeight="1" s="3">
-      <c r="C478" t="inlineStr">
+      <c r="C478" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="479" ht="15.75" customHeight="1" s="3">
-      <c r="C479" t="inlineStr">
+      <c r="C479" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="480" ht="15.75" customHeight="1" s="3">
-      <c r="C480" t="inlineStr">
+      <c r="C480" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="481" ht="15.75" customHeight="1" s="3">
-      <c r="C481" t="inlineStr">
+      <c r="C481" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="482" ht="15.75" customHeight="1" s="3">
-      <c r="C482" t="inlineStr">
+      <c r="C482" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="483" ht="15.75" customHeight="1" s="3">
-      <c r="C483" t="inlineStr">
+      <c r="C483" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="484" ht="15.75" customHeight="1" s="3">
-      <c r="C484" t="inlineStr">
+      <c r="C484" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="485" ht="15.75" customHeight="1" s="3">
-      <c r="C485" t="inlineStr">
+      <c r="C485" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="486" ht="15.75" customHeight="1" s="3">
-      <c r="C486" t="inlineStr">
+      <c r="C486" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="487" ht="15.75" customHeight="1" s="3">
-      <c r="C487" t="inlineStr">
+      <c r="C487" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="488" ht="15.75" customHeight="1" s="3">
-      <c r="C488" t="inlineStr">
+      <c r="C488" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="489" ht="15.75" customHeight="1" s="3">
-      <c r="C489" t="inlineStr">
+      <c r="C489" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="490" ht="15.75" customHeight="1" s="3">
-      <c r="C490" t="inlineStr">
+      <c r="C490" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="491" ht="15.75" customHeight="1" s="3">
-      <c r="C491" t="inlineStr">
+      <c r="C491" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="492" ht="15.75" customHeight="1" s="3">
-      <c r="C492" t="inlineStr">
+      <c r="C492" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="493" ht="15.75" customHeight="1" s="3">
-      <c r="C493" t="inlineStr">
+      <c r="C493" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="494" ht="15.75" customHeight="1" s="3">
-      <c r="C494" t="inlineStr">
+      <c r="C494" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="495" ht="15.75" customHeight="1" s="3">
-      <c r="C495" t="inlineStr">
+      <c r="C495" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="496" ht="15.75" customHeight="1" s="3">
-      <c r="C496" t="inlineStr">
+      <c r="C496" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="497" ht="15.75" customHeight="1" s="3">
-      <c r="C497" t="inlineStr">
+      <c r="C497" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="498" ht="15.75" customHeight="1" s="3">
-      <c r="C498" t="inlineStr">
+      <c r="C498" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="499" ht="15.75" customHeight="1" s="3">
-      <c r="C499" t="inlineStr">
+      <c r="C499" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="500" ht="15.75" customHeight="1" s="3">
-      <c r="C500" t="inlineStr">
+      <c r="C500" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
     <row r="501" ht="15.75" customHeight="1" s="3">
-      <c r="C501" t="inlineStr">
+      <c r="C501" s="0" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>